<commit_message>
Added PSI automation and validation enhancements
</commit_message>
<xml_diff>
--- a/output/validation_summary.xlsx
+++ b/output/validation_summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,6 +432,16 @@
           <t>Validation</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Difference</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>% Change</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -445,6 +455,12 @@
       <c r="C2" t="n">
         <v>0.6558353972375242</v>
       </c>
+      <c r="D2" t="n">
+        <v>-0.06416460276247582</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-8.911750383677198</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -458,6 +474,12 @@
       <c r="C3" t="n">
         <v>0.2346716375838014</v>
       </c>
+      <c r="D3" t="n">
+        <v>-0.1153283624161986</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-32.95096069034246</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -470,6 +492,12 @@
       </c>
       <c r="C4" t="n">
         <v>0.3116707944750483</v>
+      </c>
+      <c r="D4" t="n">
+        <v>-0.1283292055249517</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-29.16572852839811</v>
       </c>
     </row>
   </sheetData>

</xml_diff>